<commit_message>
add EKF and replace source code from D435i to D430 camera
</commit_message>
<xml_diff>
--- a/VDT_project.xlsx
+++ b/VDT_project.xlsx
@@ -5031,13 +5031,821 @@
       </c>
       <c r="V32" s="44"/>
     </row>
+    <row r="33" spans="1:22" ht="40.049999999999997" customHeight="1">
+      <c r="A33" s="21">
+        <v>30</v>
+      </c>
+      <c r="B33" s="21" t="inlineStr">
+        <is>
+          <t>GĐ1-T11</t>
+        </is>
+      </c>
+      <c r="C33" s="53" t="inlineStr">
+        <is>
+          <t>GĐ1: Setup &amp; Sim</t>
+        </is>
+      </c>
+      <c r="D33" s="21" t="inlineStr">
+        <is>
+          <t>W1</t>
+        </is>
+      </c>
+      <c r="E33" s="21" t="inlineStr">
+        <is>
+          <t>M1</t>
+        </is>
+      </c>
+      <c r="F33" s="31" t="inlineStr">
+        <is>
+          <t>Dựng Gazebo world mô phỏng H-Pad, drone, platform và vật cản</t>
+        </is>
+      </c>
+      <c r="G33" s="42" t="inlineStr">
+        <is>
+          <t>Tạo world có quadrotor PX4, H-Pad gắn ArUco trên platform chuyển động, 3–5 vật cản có khoảng cách ≥ 1,5 m và ground plane. Khai báo model/plugin pose để có ground truth và kịch bản platform chạy ≤ 1 m/s.</t>
+        </is>
+      </c>
+      <c r="H33" s="21" t="inlineStr">
+        <is>
+          <t>Tuân</t>
+        </is>
+      </c>
+      <c r="I33" s="21" t="inlineStr">
+        <is>
+          <t>Việt Anh</t>
+        </is>
+      </c>
+      <c r="J33" s="54" t="inlineStr">
+        <is>
+          <t>🔴 Critical</t>
+        </is>
+      </c>
+      <c r="K33" s="21" t="inlineStr">
+        <is>
+          <t>GĐ1-T04</t>
+        </is>
+      </c>
+      <c r="L33" s="32">
+        <v>46258</v>
+      </c>
+      <c r="M33" s="32">
+        <v>46261</v>
+      </c>
+      <c r="N33" s="32" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="O33" s="32" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="P33" s="21" t="inlineStr">
+        <is>
+          <t>⬜ Not Started</t>
+        </is>
+      </c>
+      <c r="Q33" s="43">
+        <v>0</v>
+      </c>
+      <c r="R33" s="20">
+        <f>IF(P33="✅ Done","—",MAX(0,M33-TODAY()))</f>
+        <v>0</v>
+      </c>
+      <c r="S33" s="21">
+        <v>16</v>
+      </c>
+      <c r="T33" s="44" t="inlineStr">
+        <is>
+          <t>Gazebo world + model files + scenario YAML</t>
+        </is>
+      </c>
+      <c r="U33" s="44" t="inlineStr">
+        <is>
+          <t>World khởi động lặp lại được; drone, H-Pad, vật cản và platform xuất hiện đúng frame; ground truth pose ghi được.</t>
+        </is>
+      </c>
+      <c r="V33" s="44" t="inlineStr">
+        <is>
+          <t>Simulation: Gazebo</t>
+        </is>
+      </c>
+    </row>
+    <row r="34" spans="1:22" ht="40.049999999999997" customHeight="1">
+      <c r="A34" s="21">
+        <v>31</v>
+      </c>
+      <c r="B34" s="21" t="inlineStr">
+        <is>
+          <t>GĐ1-T12</t>
+        </is>
+      </c>
+      <c r="C34" s="53" t="inlineStr">
+        <is>
+          <t>GĐ1: Setup &amp; Sim</t>
+        </is>
+      </c>
+      <c r="D34" s="21" t="inlineStr">
+        <is>
+          <t>W1</t>
+        </is>
+      </c>
+      <c r="E34" s="21" t="inlineStr">
+        <is>
+          <t>M1</t>
+        </is>
+      </c>
+      <c r="F34" s="31" t="inlineStr">
+        <is>
+          <t>Kết nối PX4 SITL–Gazebo–ROS 2 và kiểm tra luồng telemetry</t>
+        </is>
+      </c>
+      <c r="G34" s="42" t="inlineStr">
+        <is>
+          <t>Khởi chạy PX4 SITL cùng Gazebo, micro-XRCE-DDS/px4_ros_com và ROS 2 bridge. Kiểm tra /fmu/out/vehicle_odometry, vehicle_status, command/offboard và đồng bộ timestamp.</t>
+        </is>
+      </c>
+      <c r="H34" s="21" t="inlineStr">
+        <is>
+          <t>Việt Anh</t>
+        </is>
+      </c>
+      <c r="I34" s="21" t="inlineStr">
+        <is>
+          <t>Duy</t>
+        </is>
+      </c>
+      <c r="J34" s="54" t="inlineStr">
+        <is>
+          <t>🔴 Critical</t>
+        </is>
+      </c>
+      <c r="K34" s="21" t="inlineStr">
+        <is>
+          <t>GĐ1-T04, GĐ1-T11</t>
+        </is>
+      </c>
+      <c r="L34" s="32">
+        <v>46260</v>
+      </c>
+      <c r="M34" s="32">
+        <v>46263</v>
+      </c>
+      <c r="N34" s="32" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="O34" s="32" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="P34" s="21" t="inlineStr">
+        <is>
+          <t>⬜ Not Started</t>
+        </is>
+      </c>
+      <c r="Q34" s="43">
+        <v>0</v>
+      </c>
+      <c r="R34" s="20">
+        <f>IF(P34="✅ Done","—",MAX(0,M34-TODAY()))</f>
+        <v>0</v>
+      </c>
+      <c r="S34" s="21">
+        <v>14</v>
+      </c>
+      <c r="T34" s="44" t="inlineStr">
+        <is>
+          <t>Launch files + topic/TF connection checklist</t>
+        </is>
+      </c>
+      <c r="U34" s="44" t="inlineStr">
+        <is>
+          <t>PX4 arm/takeoff/land được trong SITL; ROS 2 nhận odometry ổn định ≥ 30 s; không có topic mất kết nối.</t>
+        </is>
+      </c>
+      <c r="V34" s="44" t="inlineStr">
+        <is>
+          <t>Simulation: PX4 SITL + ROS 2</t>
+        </is>
+      </c>
+    </row>
+    <row r="35" spans="1:22" ht="40.049999999999997" customHeight="1">
+      <c r="A35" s="21">
+        <v>32</v>
+      </c>
+      <c r="B35" s="21" t="inlineStr">
+        <is>
+          <t>GĐ1-T13</t>
+        </is>
+      </c>
+      <c r="C35" s="53" t="inlineStr">
+        <is>
+          <t>GĐ1: Setup &amp; Sim</t>
+        </is>
+      </c>
+      <c r="D35" s="21" t="inlineStr">
+        <is>
+          <t>W1</t>
+        </is>
+      </c>
+      <c r="E35" s="21" t="inlineStr">
+        <is>
+          <t>M1</t>
+        </is>
+      </c>
+      <c r="F35" s="31" t="inlineStr">
+        <is>
+          <t>Thiết lập RViz2 để quan sát TF, odometry, H-Pad, depth và setpoint</t>
+        </is>
+      </c>
+      <c r="G35" s="42" t="inlineStr">
+        <is>
+          <t>Tạo RViz2 config hiển thị map/odom/base_link/camera_link, marker H-Pad, pose EKF, quỹ đạo drone, obstacle point/depth và velocity/position setpoint. Kiểm tra hướng trục ENU/NED và timestamp.</t>
+        </is>
+      </c>
+      <c r="H35" s="21" t="inlineStr">
+        <is>
+          <t>Duy</t>
+        </is>
+      </c>
+      <c r="I35" s="21" t="inlineStr">
+        <is>
+          <t>Tuân</t>
+        </is>
+      </c>
+      <c r="J35" s="54" t="inlineStr">
+        <is>
+          <t>🟡 High</t>
+        </is>
+      </c>
+      <c r="K35" s="21" t="inlineStr">
+        <is>
+          <t>GĐ1-T12</t>
+        </is>
+      </c>
+      <c r="L35" s="32">
+        <v>46261</v>
+      </c>
+      <c r="M35" s="32">
+        <v>46264</v>
+      </c>
+      <c r="N35" s="32" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="O35" s="32" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="P35" s="21" t="inlineStr">
+        <is>
+          <t>⬜ Not Started</t>
+        </is>
+      </c>
+      <c r="Q35" s="43">
+        <v>0</v>
+      </c>
+      <c r="R35" s="20">
+        <f>IF(P35="✅ Done","—",MAX(0,M35-TODAY()))</f>
+        <v>0</v>
+      </c>
+      <c r="S35" s="21">
+        <v>12</v>
+      </c>
+      <c r="T35" s="44" t="inlineStr">
+        <is>
+          <t>rviz2_config + ảnh/screencast topic visualization</t>
+        </is>
+      </c>
+      <c r="U35" s="44" t="inlineStr">
+        <is>
+          <t>TF không nhảy/đứt; pose H-Pad khớp ground truth; phân biệt rõ mục tiêu, vật cản và setpoint trên RViz2.</t>
+        </is>
+      </c>
+      <c r="V35" s="44" t="inlineStr">
+        <is>
+          <t>Simulation: RViz2</t>
+        </is>
+      </c>
+    </row>
+    <row r="36" spans="1:22" ht="40.049999999999997" customHeight="1">
+      <c r="A36" s="21">
+        <v>33</v>
+      </c>
+      <c r="B36" s="21" t="inlineStr">
+        <is>
+          <t>GĐ1-T14</t>
+        </is>
+      </c>
+      <c r="C36" s="53" t="inlineStr">
+        <is>
+          <t>GĐ1: Setup &amp; Sim</t>
+        </is>
+      </c>
+      <c r="D36" s="21" t="inlineStr">
+        <is>
+          <t>W2</t>
+        </is>
+      </c>
+      <c r="E36" s="21" t="inlineStr">
+        <is>
+          <t>M1</t>
+        </is>
+      </c>
+      <c r="F36" s="31" t="inlineStr">
+        <is>
+          <t>Mô phỏng RGB-D camera, ArUco và ground truth cho pipeline vision</t>
+        </is>
+      </c>
+      <c r="G36" s="42" t="inlineStr">
+        <is>
+          <t>Cấu hình camera RGB-D/plugin hoặc ros_gz_bridge; tạo RGB, depth, camera_info và ArUco H-Pad. Đối chiếu pose PnP với ground truth ở nhiều khoảng cách/góc; kiểm tra depth masking BBox dilate 15%.</t>
+        </is>
+      </c>
+      <c r="H36" s="21" t="inlineStr">
+        <is>
+          <t>Duy</t>
+        </is>
+      </c>
+      <c r="I36" s="21" t="inlineStr">
+        <is>
+          <t>Việt Anh</t>
+        </is>
+      </c>
+      <c r="J36" s="54" t="inlineStr">
+        <is>
+          <t>🔴 Critical</t>
+        </is>
+      </c>
+      <c r="K36" s="21" t="inlineStr">
+        <is>
+          <t>GĐ1-T03, GĐ1-T11, GĐ1-T12</t>
+        </is>
+      </c>
+      <c r="L36" s="32">
+        <v>46265</v>
+      </c>
+      <c r="M36" s="32">
+        <v>46268</v>
+      </c>
+      <c r="N36" s="32" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="O36" s="32" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="P36" s="21" t="inlineStr">
+        <is>
+          <t>⬜ Not Started</t>
+        </is>
+      </c>
+      <c r="Q36" s="43">
+        <v>0</v>
+      </c>
+      <c r="R36" s="20">
+        <f>IF(P36="✅ Done","—",MAX(0,M36-TODAY()))</f>
+        <v>0</v>
+      </c>
+      <c r="S36" s="21">
+        <v>16</v>
+      </c>
+      <c r="T36" s="44" t="inlineStr">
+        <is>
+          <t>Camera/ArUco simulation launch + calibration/test dataset</t>
+        </is>
+      </c>
+      <c r="U36" s="44" t="inlineStr">
+        <is>
+          <t>Topic RGB+Depth+CameraInfo chạy liên tục; marker detect ≥ 90% frame trong vùng nhìn; sai số pose 3D &lt; 0,5 m; vùng H-Pad được mask đúng.</t>
+        </is>
+      </c>
+      <c r="V36" s="44" t="inlineStr">
+        <is>
+          <t>Simulation: RGB-D + ArUco</t>
+        </is>
+      </c>
+    </row>
+    <row r="37" spans="1:22" ht="40.049999999999997" customHeight="1">
+      <c r="A37" s="21">
+        <v>34</v>
+      </c>
+      <c r="B37" s="21" t="inlineStr">
+        <is>
+          <t>GĐ1-T15</t>
+        </is>
+      </c>
+      <c r="C37" s="53" t="inlineStr">
+        <is>
+          <t>GĐ1: Setup &amp; Sim</t>
+        </is>
+      </c>
+      <c r="D37" s="21" t="inlineStr">
+        <is>
+          <t>W2</t>
+        </is>
+      </c>
+      <c r="E37" s="21" t="inlineStr">
+        <is>
+          <t>M1</t>
+        </is>
+      </c>
+      <c r="F37" s="31" t="inlineStr">
+        <is>
+          <t>Thiết lập QGroundControl cho PX4 SITL và kiểm thử thao tác operator</t>
+        </is>
+      </c>
+      <c r="G37" s="42" t="inlineStr">
+        <is>
+          <t>Kết nối QGroundControl qua UDP; kiểm tra heartbeat, vehicle status, map/telemetry, arm/disarm, takeoff, land, mode Offboard và gán RC switch LAND/CANCEL/Kill theo kịch bản Human-in-the-Loop.</t>
+        </is>
+      </c>
+      <c r="H37" s="21" t="inlineStr">
+        <is>
+          <t>Việt Anh</t>
+        </is>
+      </c>
+      <c r="I37" s="21" t="inlineStr">
+        <is>
+          <t>Cả nhóm</t>
+        </is>
+      </c>
+      <c r="J37" s="54" t="inlineStr">
+        <is>
+          <t>🔴 Critical</t>
+        </is>
+      </c>
+      <c r="K37" s="21" t="inlineStr">
+        <is>
+          <t>GĐ1-T12</t>
+        </is>
+      </c>
+      <c r="L37" s="32">
+        <v>46266</v>
+      </c>
+      <c r="M37" s="32">
+        <v>46269</v>
+      </c>
+      <c r="N37" s="32" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="O37" s="32" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="P37" s="21" t="inlineStr">
+        <is>
+          <t>⬜ Not Started</t>
+        </is>
+      </c>
+      <c r="Q37" s="43">
+        <v>0</v>
+      </c>
+      <c r="R37" s="20">
+        <f>IF(P37="✅ Done","—",MAX(0,M37-TODAY()))</f>
+        <v>0</v>
+      </c>
+      <c r="S37" s="21">
+        <v>12</v>
+      </c>
+      <c r="T37" s="44" t="inlineStr">
+        <is>
+          <t>QGC parameter/joystick setup + operator checklist</t>
+        </is>
+      </c>
+      <c r="U37" s="44" t="inlineStr">
+        <is>
+          <t>QGC hiển thị telemetry ổn định ≥ 10 phút; operator chuyển được các mode; LAND NOW và CANCEL tạo đúng sự kiện FSM; kill/land luôn có đường thoát an toàn.</t>
+        </is>
+      </c>
+      <c r="V37" s="44" t="inlineStr">
+        <is>
+          <t>Simulation: QGroundControl</t>
+        </is>
+      </c>
+    </row>
+    <row r="38" spans="1:22" ht="40.049999999999997" customHeight="1">
+      <c r="A38" s="21">
+        <v>35</v>
+      </c>
+      <c r="B38" s="21" t="inlineStr">
+        <is>
+          <t>GĐ2-T07</t>
+        </is>
+      </c>
+      <c r="C38" s="53" t="inlineStr">
+        <is>
+          <t>GĐ2: SITL &amp; Bench</t>
+        </is>
+      </c>
+      <c r="D38" s="21" t="inlineStr">
+        <is>
+          <t>W3</t>
+        </is>
+      </c>
+      <c r="E38" s="21" t="inlineStr">
+        <is>
+          <t>M1</t>
+        </is>
+      </c>
+      <c r="F38" s="31" t="inlineStr">
+        <is>
+          <t>Kiểm thử FSM SEARCH→FOLLOW→APPROACH→LAND trên Gazebo + RViz2 + QGC</t>
+        </is>
+      </c>
+      <c r="G38" s="42" t="inlineStr">
+        <is>
+          <t>Chạy từng transition với điều kiện kiểm soát: marker mất/hiện, đủ 10 frame, LAND NOW, marker mất &gt; 3 s, alignment &lt; 0,3 m và altitude &lt; 0,5 m. Dùng QGC phát lệnh operator, RViz2 quan sát state/pose/gimbal.</t>
+        </is>
+      </c>
+      <c r="H38" s="21" t="inlineStr">
+        <is>
+          <t>Việt Anh</t>
+        </is>
+      </c>
+      <c r="I38" s="21" t="inlineStr">
+        <is>
+          <t>Duy</t>
+        </is>
+      </c>
+      <c r="J38" s="54" t="inlineStr">
+        <is>
+          <t>🔴 Critical</t>
+        </is>
+      </c>
+      <c r="K38" s="21" t="inlineStr">
+        <is>
+          <t>GĐ1-T13, GĐ1-T15, GĐ2-T03</t>
+        </is>
+      </c>
+      <c r="L38" s="32">
+        <v>46272</v>
+      </c>
+      <c r="M38" s="32">
+        <v>46275</v>
+      </c>
+      <c r="N38" s="32" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="O38" s="32" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="P38" s="21" t="inlineStr">
+        <is>
+          <t>⬜ Not Started</t>
+        </is>
+      </c>
+      <c r="Q38" s="43">
+        <v>0</v>
+      </c>
+      <c r="R38" s="20">
+        <f>IF(P38="✅ Done","—",MAX(0,M38-TODAY()))</f>
+        <v>0</v>
+      </c>
+      <c r="S38" s="21">
+        <v>16</v>
+      </c>
+      <c r="T38" s="44" t="inlineStr">
+        <is>
+          <t>FSM test matrix + rosbag + QGC/RViz2 evidence</t>
+        </is>
+      </c>
+      <c r="U38" s="44" t="inlineStr">
+        <is>
+          <t>100% transition hợp lệ; marker mất trả về đúng state; không phát setpoint nguy hiểm khi mất dữ liệu; log có timestamp vào/ra từng state.</t>
+        </is>
+      </c>
+      <c r="V38" s="44" t="inlineStr">
+        <is>
+          <t>Simulation: state-machine SIL</t>
+        </is>
+      </c>
+    </row>
+    <row r="39" spans="1:22" ht="40.049999999999997" customHeight="1">
+      <c r="A39" s="21">
+        <v>36</v>
+      </c>
+      <c r="B39" s="21" t="inlineStr">
+        <is>
+          <t>GĐ2-T08</t>
+        </is>
+      </c>
+      <c r="C39" s="53" t="inlineStr">
+        <is>
+          <t>GĐ2: SITL &amp; Bench</t>
+        </is>
+      </c>
+      <c r="D39" s="21" t="inlineStr">
+        <is>
+          <t>W3</t>
+        </is>
+      </c>
+      <c r="E39" s="21" t="inlineStr">
+        <is>
+          <t>M8/M9</t>
+        </is>
+      </c>
+      <c r="F39" s="31" t="inlineStr">
+        <is>
+          <t>Kiểm thử tích hợp FOLLOW mục tiêu động và VO-APF tránh vật cản</t>
+        </is>
+      </c>
+      <c r="G39" s="42" t="inlineStr">
+        <is>
+          <t>Chạy platform theo ít nhất 3 quỹ đạo/tốc độ, bố trí 3–5 vật cản; kiểm tra depth masking không biến H-Pad thành obstacle, lực hút/đẩy, velocity setpoint, giới hạn tốc độ và recovery khi marker bị che ngắn hạn.</t>
+        </is>
+      </c>
+      <c r="H39" s="21" t="inlineStr">
+        <is>
+          <t>Tuân</t>
+        </is>
+      </c>
+      <c r="I39" s="21" t="inlineStr">
+        <is>
+          <t>Duy</t>
+        </is>
+      </c>
+      <c r="J39" s="54" t="inlineStr">
+        <is>
+          <t>🔴 Critical</t>
+        </is>
+      </c>
+      <c r="K39" s="21" t="inlineStr">
+        <is>
+          <t>GĐ1-T11, GĐ1-T14, GĐ2-T02</t>
+        </is>
+      </c>
+      <c r="L39" s="32">
+        <v>46274</v>
+      </c>
+      <c r="M39" s="32">
+        <v>46278</v>
+      </c>
+      <c r="N39" s="32" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="O39" s="32" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="P39" s="21" t="inlineStr">
+        <is>
+          <t>⬜ Not Started</t>
+        </is>
+      </c>
+      <c r="Q39" s="43">
+        <v>0</v>
+      </c>
+      <c r="R39" s="20">
+        <f>IF(P39="✅ Done","—",MAX(0,M39-TODAY()))</f>
+        <v>0</v>
+      </c>
+      <c r="S39" s="21">
+        <v>20</v>
+      </c>
+      <c r="T39" s="44" t="inlineStr">
+        <is>
+          <t>SITL rosbag + video Gazebo/RViz2/QGC + scenario report</t>
+        </is>
+      </c>
+      <c r="U39" s="44" t="inlineStr">
+        <is>
+          <t>FOLLOW liên tục ≥ 60 s; né ≥ 3 vật cản; clearance mô phỏng &gt; 0,8 m; APF &lt; 20 ms/cycle; tracking RMSE &lt; 1,0 m.</t>
+        </is>
+      </c>
+      <c r="V39" s="44" t="inlineStr">
+        <is>
+          <t>Simulation: integrated follow/avoid</t>
+        </is>
+      </c>
+    </row>
+    <row r="40" spans="1:22" ht="40.049999999999997" customHeight="1">
+      <c r="A40" s="21">
+        <v>37</v>
+      </c>
+      <c r="B40" s="21" t="inlineStr">
+        <is>
+          <t>GĐ2-T09</t>
+        </is>
+      </c>
+      <c r="C40" s="53" t="inlineStr">
+        <is>
+          <t>GĐ2: SITL &amp; Bench</t>
+        </is>
+      </c>
+      <c r="D40" s="21" t="inlineStr">
+        <is>
+          <t>W4</t>
+        </is>
+      </c>
+      <c r="E40" s="21" t="inlineStr">
+        <is>
+          <t>M1-M10</t>
+        </is>
+      </c>
+      <c r="F40" s="31" t="inlineStr">
+        <is>
+          <t>Regression test mô phỏng và đo đủ KPI trước khi chuyển sang hardware</t>
+        </is>
+      </c>
+      <c r="G40" s="42" t="inlineStr">
+        <is>
+          <t>Tự động hóa tối thiểu 5 lần chạy cùng scenario; lưu PX4 ulog/ROS 2 bag, ảnh RViz2, video Gazebo và QGC. Tính tracking error, landing error, clearance, latency, FPS và tỷ lệ thành công; ghi rõ seed/cấu hình.</t>
+        </is>
+      </c>
+      <c r="H40" s="21" t="inlineStr">
+        <is>
+          <t>Cả nhóm</t>
+        </is>
+      </c>
+      <c r="I40" s="21" t="inlineStr">
+        <is>
+          <t>Duy</t>
+        </is>
+      </c>
+      <c r="J40" s="54" t="inlineStr">
+        <is>
+          <t>🔴 Critical</t>
+        </is>
+      </c>
+      <c r="K40" s="21" t="inlineStr">
+        <is>
+          <t>GĐ2-T07, GĐ2-T08</t>
+        </is>
+      </c>
+      <c r="L40" s="32">
+        <v>46279</v>
+      </c>
+      <c r="M40" s="32">
+        <v>46282</v>
+      </c>
+      <c r="N40" s="32" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="O40" s="32" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="P40" s="21" t="inlineStr">
+        <is>
+          <t>⬜ Not Started</t>
+        </is>
+      </c>
+      <c r="Q40" s="43">
+        <v>0</v>
+      </c>
+      <c r="R40" s="20">
+        <f>IF(P40="✅ Done","—",MAX(0,M40-TODAY()))</f>
+        <v>0</v>
+      </c>
+      <c r="S40" s="21">
+        <v>18</v>
+      </c>
+      <c r="T40" s="44" t="inlineStr">
+        <is>
+          <t>Simulation regression report + KPI CSV/plots + replay command</t>
+        </is>
+      </c>
+      <c r="U40" s="44" t="inlineStr">
+        <is>
+          <t>≥ 5 run tái lập được; full pipeline SEARCH→FOLLOW→APPROACH→LAND đạt ≥ 70%; sensor→command latency &lt; 500 ms; có lệnh replay để debug.</t>
+        </is>
+      </c>
+      <c r="V40" s="44" t="inlineStr">
+        <is>
+          <t>Gate: pass simulation before flight</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A3:V32" xr:uid="{00000000-0009-0000-0000-000001000000}"/>
+  <autoFilter ref="A3:V40" xr:uid="{00000000-0009-0000-0000-000001000000}"/>
   <mergeCells count="2">
     <mergeCell ref="A2:V2"/>
     <mergeCell ref="A1:V1"/>
   </mergeCells>
-  <conditionalFormatting sqref="P4:P32">
+  <conditionalFormatting sqref="P4:P40">
     <cfRule type="cellIs" dxfId="7" priority="1" operator="equal">
       <formula>"✅ Done"</formula>
     </cfRule>
@@ -5070,16 +5878,16 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="4">
-    <dataValidation type="list" allowBlank="1" errorTitle="Invalid Status" error="Please select a valid status" sqref="P4:P32" xr:uid="{00000000-0002-0000-0100-000000000000}">
+    <dataValidation type="list" allowBlank="1" errorTitle="Invalid Status" error="Please select a valid status" sqref="P4:P40" xr:uid="{00000000-0002-0000-0100-000000000000}">
       <formula1>"⬜ Not Started,🔵 In Progress,✅ Done,🔴 Blocked,⏰ Overdue,⏸ On Hold"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" sqref="J4:J32" xr:uid="{00000000-0002-0000-0100-000001000000}">
+    <dataValidation type="list" allowBlank="1" sqref="J4:J40" xr:uid="{00000000-0002-0000-0100-000001000000}">
       <formula1>"🔴 Critical,🟡 High,🟢 Normal,⚪ Low"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" sqref="H4:H32" xr:uid="{00000000-0002-0000-0100-000002000000}">
+    <dataValidation type="list" allowBlank="1" sqref="H4:H40" xr:uid="{00000000-0002-0000-0100-000002000000}">
       <formula1>"Duy,Tuân,Việt Anh,Cả nhóm"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" sqref="I4:I32" xr:uid="{00000000-0002-0000-0100-000003000000}">
+    <dataValidation type="list" allowBlank="1" sqref="I4:I40" xr:uid="{00000000-0002-0000-0100-000003000000}">
       <formula1>"Duy,Tuân,Việt Anh,—"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>